<commit_message>
Resolve Geant4 pkg-config from build tree, dedupe G4 link libs
</commit_message>
<xml_diff>
--- a/geometry_source/targets/rge_runs.xlsx
+++ b/geometry_source/targets/rge_runs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/opt/projects/gemc/clas12Tags/geometry_source/targets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FFEA3A8-79E7-0644-AF03-0E37D011AB0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B39D4E00-9240-454A-A450-22B82327AC3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1920" windowWidth="41120" windowHeight="24420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51440" yWindow="280" windowWidth="48220" windowHeight="27320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="47">
   <si>
     <t>Original geometry</t>
   </si>
@@ -144,6 +144,30 @@
   <si>
     <t>LD2-Cu-sol-Inb
 LD2-Cu-liq-Inb</t>
+  </si>
+  <si>
+    <t>Solid Target</t>
+  </si>
+  <si>
+    <t>Thickness</t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
+    <t>0.6x2</t>
+  </si>
+  <si>
+    <t>0.74x2</t>
+  </si>
+  <si>
+    <t>0.18x2</t>
+  </si>
+  <si>
+    <t>0.15x2</t>
+  </si>
+  <si>
+    <t>0.07x2</t>
   </si>
 </sst>
 </file>
@@ -649,7 +673,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="7">
-        <v>20506</v>
+        <v>20014</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="13" x14ac:dyDescent="0.15">
@@ -671,8 +695,8 @@
       <c r="F3" s="5">
         <v>0</v>
       </c>
-      <c r="G3" s="7">
-        <v>20014</v>
+      <c r="G3" s="11">
+        <v>20021</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13" x14ac:dyDescent="0.15">
@@ -695,7 +719,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="7">
-        <v>20070</v>
+        <v>20035</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13" x14ac:dyDescent="0.15">
@@ -717,8 +741,8 @@
       <c r="F5" s="5">
         <v>0</v>
       </c>
-      <c r="G5" s="7">
-        <v>20035</v>
+      <c r="G5" s="11">
+        <v>20041</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13" x14ac:dyDescent="0.15">
@@ -740,8 +764,8 @@
       <c r="F6" s="9">
         <v>0</v>
       </c>
-      <c r="G6" s="11">
-        <v>20507</v>
+      <c r="G6" s="7">
+        <v>20070</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="13" x14ac:dyDescent="0.15">
@@ -764,7 +788,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="11">
-        <v>20269</v>
+        <v>20074</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -787,7 +811,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="7">
-        <v>20435</v>
+        <v>20131</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -810,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="11">
-        <v>20021</v>
+        <v>20177</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -833,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="7">
-        <v>20131</v>
+        <v>20232</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -855,8 +879,8 @@
       <c r="F11" s="5">
         <v>0</v>
       </c>
-      <c r="G11" s="7">
-        <v>20508</v>
+      <c r="G11" s="11">
+        <v>20269</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -878,8 +902,8 @@
       <c r="F12" s="9">
         <v>0</v>
       </c>
-      <c r="G12" s="11">
-        <v>20177</v>
+      <c r="G12" s="7">
+        <v>20282</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -902,7 +926,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="11">
-        <v>20041</v>
+        <v>20331</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -924,8 +948,8 @@
       <c r="F14" s="9">
         <v>0</v>
       </c>
-      <c r="G14" s="11">
-        <v>20074</v>
+      <c r="G14" s="7">
+        <v>20435</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -947,8 +971,8 @@
       <c r="F15" s="5">
         <v>0</v>
       </c>
-      <c r="G15" s="7">
-        <v>20232</v>
+      <c r="G15" s="11">
+        <v>20494</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -971,7 +995,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="7">
-        <v>20282</v>
+        <v>20506</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -994,7 +1018,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="11">
-        <v>20494</v>
+        <v>20507</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -1016,8 +1040,8 @@
       <c r="F18" s="9">
         <v>0</v>
       </c>
-      <c r="G18" s="11">
-        <v>20520</v>
+      <c r="G18" s="7">
+        <v>20508</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28" x14ac:dyDescent="0.15">
@@ -1040,7 +1064,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="15">
-        <v>20331</v>
+        <v>20520</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1062,54 +1086,90 @@
       <c r="G21" s="16"/>
     </row>
     <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="16"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="16"/>
+      <c r="A22" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>40</v>
+      </c>
       <c r="D22" s="16"/>
       <c r="E22" s="16"/>
       <c r="F22" s="16"/>
       <c r="G22" s="16"/>
     </row>
     <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="16"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="16"/>
+      <c r="A23" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="16">
+        <v>-1.5</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>42</v>
+      </c>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
       <c r="G23" s="16"/>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="16"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
+      <c r="A24" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="16">
+        <v>-1.5</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>43</v>
+      </c>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
       <c r="G24" s="16"/>
     </row>
     <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="16"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
+      <c r="A25" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="16">
+        <v>-1.5</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>44</v>
+      </c>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
       <c r="G25" s="16"/>
     </row>
     <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="16"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
+      <c r="A26" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="16">
+        <v>-1.5</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>45</v>
+      </c>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>
       <c r="F26" s="16"/>
       <c r="G26" s="16"/>
     </row>
     <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
+      <c r="A27" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" s="16">
+        <v>-1.5</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>46</v>
+      </c>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
@@ -9873,8 +9933,8 @@
       <c r="G1000" s="16"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G1000">
-    <sortCondition ref="D2:D1000"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G2:G1000">
+    <sortCondition ref="G2:G1000"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>